<commit_message>
Align category and request-type dropdowns with the client's item list
Categories follow the client's work-item groups; request type is the
3-choice used on calls (repair/replace, leak, urgent).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019yfLUgJbEwFDH66CcmKaRq
</commit_message>
<xml_diff>
--- a/こころ住設_案件管理シート_叩き台.xlsx
+++ b/こころ住設_案件管理シート_叩き台.xlsx
@@ -916,7 +916,7 @@
       </c>
       <c r="P3" s="17" t="inlineStr">
         <is>
-          <t>交換</t>
+          <t>交換・修理</t>
         </is>
       </c>
       <c r="Q3" s="17" t="n"/>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="P4" s="17" t="inlineStr">
         <is>
-          <t>交換</t>
+          <t>交換・修理</t>
         </is>
       </c>
       <c r="Q4" s="17" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="P5" s="17" t="inlineStr">
         <is>
-          <t>水漏れ・詰まり</t>
+          <t>緊急対応</t>
         </is>
       </c>
       <c r="Q5" s="17" t="n"/>
@@ -1292,10 +1292,10 @@
       <formula1>選択肢!$I$2:$I$6</formula1>
     </dataValidation>
     <dataValidation sqref="O3:O1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>選択肢!$J$2:$J$9</formula1>
+      <formula1>選択肢!$J$2:$J$10</formula1>
     </dataValidation>
     <dataValidation sqref="P3:P1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>選択肢!$K$2:$K$5</formula1>
+      <formula1>選択肢!$K$2:$K$4</formula1>
     </dataValidation>
     <dataValidation sqref="R3:R1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>選択肢!$L$2:$L$3</formula1>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="F16" s="20" t="inlineStr">
         <is>
-          <t>トイレ／キッチン／浴室・給湯器／洗面・蛇口／換気扇／電気／ガスコンロ・食洗機／その他（分類は木場さんが叩き台を作成中）</t>
+          <t>トイレ／キッチン／給湯器／換気扇／風呂／その他水回り／水栓・蛇口／電気関係／その他（清水様の工事可能品目の区分）</t>
         </is>
       </c>
     </row>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="F17" s="20" t="inlineStr">
         <is>
-          <t>交換／修理／水漏れ・詰まり／その他</t>
+          <t>交換・修理／水漏れ／緊急対応。換気扇・電気関係は交換・修理のみ</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1915,7 @@
       </c>
       <c r="F18" s="20" t="inlineStr">
         <is>
-          <t>例：壁紙・床の張り替えも希望</t>
+          <t>お客様が品目まで話した場合にメモ（例：ウォシュレット交換、手すり設置も）</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q9"/>
+  <dimension ref="A1:Q10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>交換</t>
+          <t>交換・修理</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>修理</t>
+          <t>水漏れ</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -2893,12 +2893,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>浴室・給湯器</t>
+          <t>給湯器</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>水漏れ・詰まり</t>
+          <t>緊急対応</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -2945,12 +2945,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>洗面・蛇口</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>その他</t>
+          <t>換気扇</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -2977,7 +2972,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>換気扇</t>
+          <t>風呂</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -2994,7 +2989,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>電気</t>
+          <t>その他水回り</t>
         </is>
       </c>
     </row>
@@ -3006,7 +3001,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>ガスコンロ・食洗機</t>
+          <t>水栓・蛇口</t>
         </is>
       </c>
     </row>
@@ -3017,6 +3012,13 @@
         </is>
       </c>
       <c r="J9" t="inlineStr">
+        <is>
+          <t>電気関係</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="J10" t="inlineStr">
         <is>
           <t>その他</t>
         </is>

</xml_diff>